<commit_message>
feat: motor de Matching D3-D6, fator multiplicador e propagacao de datas pra BC3
- Adiciona D3 (consolidacao N-para-1), D4 (integridade de nota), D5
  (ultimo recurso por similaridade) e D6 (valor + desempate por texto)
  ao motor de Matching, alem da familia de aprendizado A1-A5.
- Renumera a familia D pra refletir a ordem real de execucao
  (D1-D2-D3-D4-D5-D6, com a familia A rodando entre D2 e D3).
- Adiciona FATOR_MULTIPLICADOR_SUGERIDO (sinaliza divergencia de
  unidade/embalagem quando VL_ITEM bate entre XML e SPED), propagado
  tambem pro dicionario de aprendizado A1-A5.
- Propaga DT_E_S/DT_FIN (datas da BC1) pra BC3, com o mesmo tratamento
  de COD_ITEM_DECLARACAO/DESCR_ITEM_DECLARACAO (sentinela 'nd'/'nm',
  heranca via dicionario de aprendizado) -- alicerce do Estagio 4.
- REGRAS_MATCHING.md/TIPOS_MATCHING_RESUMO.md atualizados como fonte
  unica dos criterios de cada tipo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TIPOS_MATCHING_TP_ALEXANDRE.xlsx
+++ b/TIPOS_MATCHING_TP_ALEXANDRE.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="270" yWindow="525" windowWidth="13095" windowHeight="5070" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tipos de Matching" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tipos de Matching" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="145621" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,12 +25,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -43,20 +45,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,17 +72,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="FFB0B0B0"/>
       </left>
       <right style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="FFB0B0B0"/>
       </right>
       <top style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="FFB0B0B0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="FFB0B0B0"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -103,7 +106,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -466,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -509,7 +512,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -539,7 +542,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -569,7 +572,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
@@ -599,7 +602,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
@@ -659,7 +662,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
@@ -689,7 +692,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
@@ -719,176 +722,278 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>D3 (integridade)</t>
+          <t>D3 (consolidacao N-para-1)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Restringe às CHV_NFE íntegras (mesma contagem de itens e mesma soma de VL_ITEM da nota) e casa 1-para-1 por similaridade de descrição normalizada</t>
+          <t>Varios itens do XML somados numa unica linha consolidada/sortido do SPED: cobertura do radical da descricao do SPED nos itens do XML, por token e ponderada por raridade (idf), + soma exata de VL_ITEM do grupo</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>0,70</t>
+          <t>0,60 (cobertura)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sim (dentro das notas íntegras)</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>nd/nm restantes após A5</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>nd/nm restantes apos A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>D4 (último recurso)</t>
+          <t>D4 (integridade)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>Restringe às CHV_NFE íntegras (mesma contagem de itens e mesma soma de VL_ITEM da nota) e casa 1-para-1 por similaridade de descrição normalizada</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>0,70</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Sim (dentro das notas íntegras)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>nd/nm restantes apos D3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>D5 (ultimo recurso)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>Só similaridade de descrição normalizada, 1-para-1, sem GTIN, valor ou integridade de nota</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>0,70</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>nd/nm restantes após D3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>nd/nm restantes apos D4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="105" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>D6 (valor + desempate por texto)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Dentro da mesma CHV_NFE (sem exigir nota integra), casa por VALOR identico; se o valor empatar (2+ itens com o mesmo valor em qualquer lado), desempata por similaridade de descricao normalizada so entre os itens empatados nesse valor -- so descarta (sem match) se a similaridade tambem empatar (excecao: duplicatas identicas nos dois lados -- mesma descricao repetida -- confirmam mesmo com empate, pois o empate e so de posicao, nao de conteudo)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>sem limiar de valor; desempate por similaridade sem limiar minimo</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>nd/nm restantes apos D5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>ND (Não Declarado)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>A CHV_NFE inteira não aparece na BC1</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Status, não critério de match</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>NM (Não Match/Sem Match)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>A CHV_NFE existe na BC1, mas o item não passou nem no D1 nem no D2</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Status, não critério de match</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Legenda:</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Amarelo = família Aprendizado / A (dicionário histórico, não exige mesma CHV_NFE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Verde = status (não é critério de match)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Numeração renomeada em 2026-07-09: Tipo 1-&gt;D1, Tipo 2-&gt;D2, Tipo 3-&gt;A1, Tipo 3.1-&gt;A2, Tipo 3.2-&gt;A3, Tipo 3.3-&gt;A4, Tipo 3.4-&gt;A5, Tipo 4-&gt;D3, Tipo 5-&gt;D4 (ver HIERARQUIA_TIPOS_TP_ALEXANDRE_vs_TP_IA.md)</t>
+          <t>Amarelo = família Aprendizado / A (dicionário histórico, não exige mesma CHV_NFE)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>"Descrição normalizada" = maiúsculas, sem caracteres especiais (#, /, -, ., etc.) — implementado em 2026-07-09, reduziu NM em 21-70% nas 3 operações</t>
+          <t>Verde = status (não é critério de match)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ordem mantida (avaliado e descartado inverter D3/D4 pra antes da família A — pioraria os resultados)</t>
+          <t>Numeração renomeada em 2026-07-09: Tipo 1-&gt;D1, Tipo 2-&gt;D2, Tipo 3-&gt;A1, Tipo 3.1-&gt;A2, Tipo 3.2-&gt;A3, Tipo 3.3-&gt;A4, Tipo 3.4-&gt;A5, Tipo 4-&gt;D3, Tipo 5-&gt;D4 (ver HIERARQUIA_TIPOS_TP_ALEXANDRE_vs_TP_IA.md)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>"Descrição normalizada" = maiúsculas, sem caracteres especiais (#, /, -, ., etc.) — implementado em 2026-07-09, reduziu NM em 21-70% nas 3 operações</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ordem mantida (avaliado e descartado inverter D3/D4 pra antes da família A — pioraria os resultados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Fonte: REGRAS_MATCHING.md (atualizar a planilha junto, se as regras mudarem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>D5 adicionado em 2026-07-10 (revisita e substitui a ideia de "Tipo 6" descartada em 2026-07-09) — unico tipo N-para-1; roda antes do D3/D4 para nao perder a linha consolidada do SPED para um match 1-para-1 por coincidencia de texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>D6 (valor + desempate por texto em caso de empate) implementado em 2026-07-10, a pedido do usuario: valor unico confirma direto; valor empatado desempata por similaridade de descricao so entre os empatados, descartando apenas se a similaridade tambem empatar. NAO exige mais nota integra (removido no mesmo dia): A1-A5 nao consome BC1, entao a integridade da nota ficava poluida por linhas ja usadas por aprendizado pra outros itens, bloqueando pares isoladamente reconciliaveis. Validado na base real do geraldo: D6 total foi de 1.721 para 2.477 itens</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>D6: excecao de duplicatas identicas adicionada em 2026-07-10 (mesmo dia), a partir de caso real na operacao PB2 (CHV_NFE 25250819447771000150550010000128321164733115): 2 itens identicos do XML (mesma descricao e valor) empatavam contra 2 itens identicos do SPED e eram descartados sem necessidade -- agora confirma quando o empate e so de posicao (mesmo par de descricoes), nao de conteudo. Geraldo: D6 de 2.477 para 2.525; PB2: D6 de 15 para 17 (NM de 2 para 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>FATOR_MULTIPLICADOR_SUGERIDO (coluna nova na BC3, nao e um Tipo): adicionado em 2026-07-11, a pedido do usuario. Quando VL_ITEM bate entre XML e SPED (D1/D2/D3/D4/D6, nunca D5), calcula _VALOR_UNIT_ORIGINAL (unitario XML) / VALOR_UNITARIO_DECLARACAO (unitario SPED, novo campo derivado na BC1 como VL_ITEM/QTD). Sinaliza divergencia de unidade/embalagem (fator = N inteiro = provavel caixa/fardo de N unidades). Propagado pro A1-A5 via dicionario de aprendizado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>FATOR_MULTIPLICADOR_SUGERIDO: normalizacao de ruido de arredondamento adicionada em 2026-07-11 (mesmo dia), a partir de caso real na operacao PB2 (CHV_NFE 25251047508411114402552000000087151002911336, item CARNE DE SOL CX MOLE KG, vendido por peso): fator cru vinha 1,0001 em vez de 1,0 exato por arredondamento em cascata (SPED so grava QTD/VL_ITEM, nao o unitario). Fator dentro de 1% do inteiro mais proximo e arredondado pra esse inteiro; fora da tolerancia, mantem o valor calculado -- esse residuo sinaliza divergencia real (nao so embalagem), candidato a revisao manual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Renumeracao em 2026-07-11 (mesmo dia), a pedido do usuario: a familia D nao batia mais com a ordem de execucao desde a criacao do D5/consolidacao em 2026-07-10 (rodava antes do D3/D4, apesar do numero maior). Renomeado: D5(consolidacao)-&gt;D3, D3(integridade)-&gt;D4, D4(ultimo recurso)-&gt;D5. D1, D2, D6 e a familia A nao mudam. Ordem de execucao agora e literal: D1 -&gt; D2 -&gt; A1-A5 -&gt; D3 -&gt; D4 -&gt; D5 -&gt; D6. Criterios/limiares/ordem real nao mudaram, so os nomes -- inclusive os valores gravados em MATCH_TIPO. Re-persistido nas 3 operacoes reais.</t>
         </is>
       </c>
     </row>

</xml_diff>